<commit_message>
Excel: add source hyperlinks + eRank and PrintKK rows in Proxy tab
- ShelfTrend, accio.com, Nova One Advisor, eRank, PrintKK.com all linked in Source column
- Added eRank 2025 row: #215 keyword, +57% Nov-Dec growth
- Added PrintKK row: 50-unit MOQ, no taxonomy, no FTC compliance

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/Printify_Leather_PRD_Workbook.xlsx
+++ b/output/Printify_Leather_PRD_Workbook.xlsx
@@ -26,7 +26,7 @@
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0&quot;K&quot;"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -113,6 +113,12 @@
       <name val="Calibri"/>
       <color rgb="00B45309"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="002B5A18"/>
+      <sz val="9"/>
+      <u val="single"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -283,7 +289,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="110">
+  <cellXfs count="112">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -455,6 +461,12 @@
     <xf numFmtId="0" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -464,7 +476,7 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -482,7 +494,7 @@
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -581,7 +593,7 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -592,10 +604,10 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -952,7 +964,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Proxy Data &amp; Metrics'!B30</f>
+              <f>'Proxy Data &amp; Metrics'!B32</f>
             </strRef>
           </tx>
           <spPr>
@@ -973,12 +985,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Proxy Data &amp; Metrics'!$A$31:$A$34</f>
+              <f>'Proxy Data &amp; Metrics'!$A$33:$A$36</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Proxy Data &amp; Metrics'!$B$31:$B$34</f>
+              <f>'Proxy Data &amp; Metrics'!$B$33:$B$36</f>
             </numRef>
           </val>
         </ser>
@@ -987,7 +999,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Proxy Data &amp; Metrics'!C30</f>
+              <f>'Proxy Data &amp; Metrics'!C32</f>
             </strRef>
           </tx>
           <spPr>
@@ -1008,12 +1020,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Proxy Data &amp; Metrics'!$A$31:$A$34</f>
+              <f>'Proxy Data &amp; Metrics'!$A$33:$A$36</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Proxy Data &amp; Metrics'!$C$31:$C$34</f>
+              <f>'Proxy Data &amp; Metrics'!$C$33:$C$36</f>
             </numRef>
           </val>
         </ser>
@@ -1022,7 +1034,7 @@
           <order val="2"/>
           <tx>
             <strRef>
-              <f>'Proxy Data &amp; Metrics'!D30</f>
+              <f>'Proxy Data &amp; Metrics'!D32</f>
             </strRef>
           </tx>
           <spPr>
@@ -1043,12 +1055,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Proxy Data &amp; Metrics'!$A$31:$A$34</f>
+              <f>'Proxy Data &amp; Metrics'!$A$33:$A$36</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Proxy Data &amp; Metrics'!$D$31:$D$34</f>
+              <f>'Proxy Data &amp; Metrics'!$D$33:$D$36</f>
             </numRef>
           </val>
         </ser>
@@ -1612,7 +1624,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>35</row>
+      <row>37</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7200000" cy="3960000"/>
@@ -3747,7 +3759,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3821,7 +3833,7 @@
           <t>#215 top search term · $35–$70 AOV · 125%+ CTR</t>
         </is>
       </c>
-      <c r="D5" s="10" t="inlineStr">
+      <c r="D5" s="59" t="inlineStr">
         <is>
           <t>ShelfTrend 2025</t>
         </is>
@@ -3853,7 +3865,7 @@
           <t>$130K–$270K / week</t>
         </is>
       </c>
-      <c r="D6" s="18" t="inlineStr">
+      <c r="D6" s="60" t="inlineStr">
         <is>
           <t>ShelfTrend 2025</t>
         </is>
@@ -3885,7 +3897,7 @@
           <t>BULLIANT wallet — 8,365 units / month (BSR rank)</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="D7" s="59" t="inlineStr">
         <is>
           <t>accio.com 2025</t>
         </is>
@@ -3917,7 +3929,7 @@
           <t>$54.26B total · 6.7% CAGR · custom/POD ~$2B addressable (est.)</t>
         </is>
       </c>
-      <c r="D8" s="18" t="inlineStr">
+      <c r="D8" s="60" t="inlineStr">
         <is>
           <t>Nova One Advisor 2025</t>
         </is>
@@ -4000,117 +4012,141 @@
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
+          <t>"leather" Etsy USA keyword rank · seasonal growth</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Etsy USA</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>#215 top keyword · +57% search volume growth Nov–Dec (gifting peak)</t>
+        </is>
+      </c>
+      <c r="D11" s="59" t="inlineStr">
+        <is>
+          <t>eRank 2025</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>Seasonal signal; search ≠ confirmed purchase intent</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="33" t="inlineStr">
+        <is>
+          <t>PrintKK competitor — genuine leather MOQ</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>PrintKK</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>50-unit minimum order · no taxonomy fields · no FTC compliance</t>
+        </is>
+      </c>
+      <c r="D12" s="60" t="inlineStr">
+        <is>
+          <t>Public pricing (printKK.com)</t>
+        </is>
+      </c>
+      <c r="E12" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>Direct-observation gap: Printify 1-unit MOQ = structural differentiator</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
           <t>High-GMV Decorators routing to PrintKK / direct</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>Outreach assumption</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
+      <c r="C13" s="10" t="inlineStr">
         <is>
           <t>Unconfirmed — PoC LOI outreach will validate</t>
         </is>
       </c>
-      <c r="D11" s="10" t="inlineStr">
+      <c r="D13" s="10" t="inlineStr">
         <is>
           <t>PM hypothesis</t>
         </is>
       </c>
-      <c r="E11" s="54" t="inlineStr">
+      <c r="E13" s="54" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F11" s="10" t="inlineStr">
+      <c r="F13" s="10" t="inlineStr">
         <is>
           <t>PoC Gate 0 is the first hard data point</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="5" customHeight="1"/>
-    <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="3" t="inlineStr">
+    <row r="15" ht="5" customHeight="1"/>
+    <row r="16" ht="16" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>2. Pilot Math — How the Base Case Is Calculated</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="28" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>Variable</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>Formula / Explanation</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr"/>
-      <c r="E15" s="4" t="inlineStr"/>
-      <c r="F15" s="4" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="9" t="inlineStr">
-        <is>
-          <t>Pilot Decorators</t>
-        </is>
-      </c>
-      <c r="B16" s="27" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="C16" s="59" t="inlineStr">
-        <is>
-          <t>PoC outreach: 50 existing Printify customers → ~10% conversion → ≥ 5 LOIs</t>
-        </is>
-      </c>
-      <c r="D16" s="36" t="n"/>
-      <c r="E16" s="36" t="n"/>
-      <c r="F16" s="37" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="33" t="inlineStr">
-        <is>
-          <t>SKUs per Decorator</t>
-        </is>
-      </c>
-      <c r="B17" s="60" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="C17" s="61" t="inlineStr">
-        <is>
-          <t>Each Decorator lists 30 products (wallets, bags, journals, belts)</t>
-        </is>
-      </c>
-      <c r="D17" s="36" t="n"/>
-      <c r="E17" s="36" t="n"/>
-      <c r="F17" s="37" t="n"/>
+      <c r="D17" s="4" t="inlineStr"/>
+      <c r="E17" s="4" t="inlineStr"/>
+      <c r="F17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>Total pilot SKUs</t>
+          <t>Pilot Decorators</t>
         </is>
       </c>
       <c r="B18" s="27" t="inlineStr">
         <is>
-          <t>150</t>
-        </is>
-      </c>
-      <c r="C18" s="59" t="inlineStr">
-        <is>
-          <t>5 × 30 = 150 · minimum for marketplace algorithm indexing</t>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C18" s="61" t="inlineStr">
+        <is>
+          <t>PoC outreach: 50 existing Printify customers → ~10% conversion → ≥ 5 LOIs</t>
         </is>
       </c>
       <c r="D18" s="36" t="n"/>
@@ -4120,17 +4156,17 @@
     <row r="19">
       <c r="A19" s="33" t="inlineStr">
         <is>
-          <t>Platform margin / order</t>
-        </is>
-      </c>
-      <c r="B19" s="30" t="inlineStr">
-        <is>
-          <t>$8</t>
-        </is>
-      </c>
-      <c r="C19" s="61" t="inlineStr">
-        <is>
-          <t>Premium leather AOV $45–65 supports $8 vs. standard $5 for apparel</t>
+          <t>SKUs per Decorator</t>
+        </is>
+      </c>
+      <c r="B19" s="62" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="C19" s="63" t="inlineStr">
+        <is>
+          <t>Each Decorator lists 30 products (wallets, bags, journals, belts)</t>
         </is>
       </c>
       <c r="D19" s="36" t="n"/>
@@ -4140,17 +4176,17 @@
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>Orders/SKU/month (base)</t>
+          <t>Total pilot SKUs</t>
         </is>
       </c>
       <c r="B20" s="27" t="inlineStr">
         <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="C20" s="59" t="inlineStr">
-        <is>
-          <t>Top-quartile Etsy leather sellers proxy (kill threshold = &lt; 15 at Month 2)</t>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="C20" s="61" t="inlineStr">
+        <is>
+          <t>5 × 30 = 150 · minimum for marketplace algorithm indexing</t>
         </is>
       </c>
       <c r="D20" s="36" t="n"/>
@@ -4160,17 +4196,17 @@
     <row r="21">
       <c r="A21" s="33" t="inlineStr">
         <is>
-          <t>Monthly orders (pilot)</t>
-        </is>
-      </c>
-      <c r="B21" s="60" t="inlineStr">
-        <is>
-          <t>3,000</t>
-        </is>
-      </c>
-      <c r="C21" s="61" t="inlineStr">
-        <is>
-          <t>150 SKUs × 20 orders = 3,000 orders/month</t>
+          <t>Platform margin / order</t>
+        </is>
+      </c>
+      <c r="B21" s="30" t="inlineStr">
+        <is>
+          <t>$8</t>
+        </is>
+      </c>
+      <c r="C21" s="63" t="inlineStr">
+        <is>
+          <t>Premium leather AOV $45–65 supports $8 vs. standard $5 for apparel</t>
         </is>
       </c>
       <c r="D21" s="36" t="n"/>
@@ -4180,17 +4216,17 @@
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>Monthly margin (pilot)</t>
-        </is>
-      </c>
-      <c r="B22" s="32" t="inlineStr">
-        <is>
-          <t>$24,000</t>
-        </is>
-      </c>
-      <c r="C22" s="59" t="inlineStr">
-        <is>
-          <t>3,000 orders × $8 = $24K/month during pilot phase</t>
+          <t>Orders/SKU/month (base)</t>
+        </is>
+      </c>
+      <c r="B22" s="27" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="C22" s="61" t="inlineStr">
+        <is>
+          <t>Top-quartile Etsy leather sellers proxy (kill threshold = &lt; 15 at Month 2)</t>
         </is>
       </c>
       <c r="D22" s="36" t="n"/>
@@ -4200,17 +4236,17 @@
     <row r="23">
       <c r="A23" s="33" t="inlineStr">
         <is>
-          <t>Monthly margin (full scale)</t>
-        </is>
-      </c>
-      <c r="B23" s="30" t="inlineStr">
-        <is>
-          <t>$150,000</t>
-        </is>
-      </c>
-      <c r="C23" s="61" t="inlineStr">
-        <is>
-          <t>10 Decorators × 150 SKUs × 20 orders × $8 = $150K/month</t>
+          <t>Monthly orders (pilot)</t>
+        </is>
+      </c>
+      <c r="B23" s="62" t="inlineStr">
+        <is>
+          <t>3,000</t>
+        </is>
+      </c>
+      <c r="C23" s="63" t="inlineStr">
+        <is>
+          <t>150 SKUs × 20 orders = 3,000 orders/month</t>
         </is>
       </c>
       <c r="D23" s="36" t="n"/>
@@ -4220,17 +4256,17 @@
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>Annual run-rate (base)</t>
+          <t>Monthly margin (pilot)</t>
         </is>
       </c>
       <c r="B24" s="32" t="inlineStr">
         <is>
-          <t>$1,800,000</t>
-        </is>
-      </c>
-      <c r="C24" s="59" t="inlineStr">
-        <is>
-          <t>$150K/month × 12 months</t>
+          <t>$24,000</t>
+        </is>
+      </c>
+      <c r="C24" s="61" t="inlineStr">
+        <is>
+          <t>3,000 orders × $8 = $24K/month during pilot phase</t>
         </is>
       </c>
       <c r="D24" s="36" t="n"/>
@@ -4240,17 +4276,17 @@
     <row r="25">
       <c r="A25" s="33" t="inlineStr">
         <is>
-          <t>Total investment</t>
+          <t>Monthly margin (full scale)</t>
         </is>
       </c>
       <c r="B25" s="30" t="inlineStr">
         <is>
-          <t>$340,000</t>
-        </is>
-      </c>
-      <c r="C25" s="61" t="inlineStr">
-        <is>
-          <t>PoC $0 + Design Sprint $20K + MVP 1 $80K + MVP 2 $120K + MVP 3 $120K</t>
+          <t>$150,000</t>
+        </is>
+      </c>
+      <c r="C25" s="63" t="inlineStr">
+        <is>
+          <t>10 Decorators × 150 SKUs × 20 orders × $8 = $150K/month</t>
         </is>
       </c>
       <c r="D25" s="36" t="n"/>
@@ -4260,152 +4296,200 @@
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>Payback period (base)</t>
+          <t>Annual run-rate (base)</t>
         </is>
       </c>
       <c r="B26" s="32" t="inlineStr">
         <is>
-          <t>~15–17 months</t>
-        </is>
-      </c>
-      <c r="C26" s="59" t="inlineStr">
-        <is>
-          <t>$340K investment ÷ ramping margin — reaches positive at ~Month 15–17</t>
+          <t>$1,800,000</t>
+        </is>
+      </c>
+      <c r="C26" s="61" t="inlineStr">
+        <is>
+          <t>$150K/month × 12 months</t>
         </is>
       </c>
       <c r="D26" s="36" t="n"/>
       <c r="E26" s="36" t="n"/>
       <c r="F26" s="37" t="n"/>
     </row>
-    <row r="28" ht="24" customHeight="1">
-      <c r="A28" s="34" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="33" t="inlineStr">
+        <is>
+          <t>Total investment</t>
+        </is>
+      </c>
+      <c r="B27" s="30" t="inlineStr">
+        <is>
+          <t>$340,000</t>
+        </is>
+      </c>
+      <c r="C27" s="63" t="inlineStr">
+        <is>
+          <t>PoC $0 + Design Sprint $20K + MVP 1 $80K + MVP 2 $120K + MVP 3 $120K</t>
+        </is>
+      </c>
+      <c r="D27" s="36" t="n"/>
+      <c r="E27" s="36" t="n"/>
+      <c r="F27" s="37" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>Payback period (base)</t>
+        </is>
+      </c>
+      <c r="B28" s="32" t="inlineStr">
+        <is>
+          <t>~15–17 months</t>
+        </is>
+      </c>
+      <c r="C28" s="61" t="inlineStr">
+        <is>
+          <t>$340K investment ÷ ramping margin — reaches positive at ~Month 15–17</t>
+        </is>
+      </c>
+      <c r="D28" s="36" t="n"/>
+      <c r="E28" s="36" t="n"/>
+      <c r="F28" s="37" t="n"/>
+    </row>
+    <row r="30" ht="24" customHeight="1">
+      <c r="A30" s="34" t="inlineStr">
         <is>
           <t>⚠ All proxy data from public sources (ShelfTrend, accio.com, Nova One Advisor, 2025). PoC LOIs and supplier SLAs are the first real data points — Gate 0 validates or kills the initiative before any engineering spend.</t>
         </is>
-      </c>
-    </row>
-    <row r="30" customHeight="1">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Timepoint</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Conservative (8/SKU)</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Base Case (20/SKU)</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Optimistic (50/SKU)</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" customHeight="1">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>W16 Shopify G1</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>3</v>
-      </c>
-      <c r="C31" t="n">
-        <v>8</v>
-      </c>
-      <c r="D31" t="n">
-        <v>14</v>
       </c>
     </row>
     <row r="32" customHeight="1">
       <c r="A32" t="inlineStr">
         <is>
-          <t>M0 Launch</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>2</v>
-      </c>
-      <c r="C32" t="n">
-        <v>4</v>
-      </c>
-      <c r="D32" t="n">
-        <v>5</v>
+          <t>Timepoint</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Conservative (8/SKU)</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Base Case (20/SKU)</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Optimistic (50/SKU)</t>
+        </is>
       </c>
     </row>
     <row r="33" customHeight="1">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Month 1</t>
+          <t>W16 Shopify G1</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C33" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="D33" t="n">
-        <v>35</v>
+        <v>14</v>
       </c>
     </row>
     <row r="34" customHeight="1">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Month 2 ◆</t>
+          <t>M0 Launch</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="C34" t="n">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="D34" t="n">
-        <v>50</v>
+        <v>5</v>
       </c>
     </row>
     <row r="35" customHeight="1">
       <c r="A35" t="inlineStr">
         <is>
+          <t>Month 1</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>6</v>
+      </c>
+      <c r="C35" t="n">
+        <v>15</v>
+      </c>
+      <c r="D35" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="36" customHeight="1">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Month 2 ◆</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>8</v>
+      </c>
+      <c r="C36" t="n">
+        <v>22</v>
+      </c>
+      <c r="D36" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="37" customHeight="1">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>Month 3</t>
         </is>
       </c>
-      <c r="B35" t="n">
+      <c r="B37" t="n">
         <v>8</v>
       </c>
-      <c r="C35" t="n">
+      <c r="C37" t="n">
         <v>25</v>
       </c>
-      <c r="D35" t="n">
+      <c r="D37" t="n">
         <v>60</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
     <mergeCell ref="C22:F22"/>
+    <mergeCell ref="A16:F16"/>
     <mergeCell ref="C18:F18"/>
-    <mergeCell ref="C17:F17"/>
+    <mergeCell ref="A30:F30"/>
     <mergeCell ref="C23:F23"/>
-    <mergeCell ref="A28:F28"/>
-    <mergeCell ref="A14:F14"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="C20:F20"/>
     <mergeCell ref="C26:F26"/>
+    <mergeCell ref="C27:F27"/>
     <mergeCell ref="C21:F21"/>
-    <mergeCell ref="C16:F16"/>
     <mergeCell ref="C25:F25"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="C19:F19"/>
     <mergeCell ref="C24:F24"/>
+    <mergeCell ref="C28:F28"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId6"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
 </worksheet>
 </file>
 
@@ -4456,7 +4540,7 @@
       </c>
     </row>
     <row r="4" ht="52" customHeight="1">
-      <c r="A4" s="62" t="inlineStr">
+      <c r="A4" s="64" t="inlineStr">
         <is>
           <t>Decorators serving the USA personalized gifting market ($40–$80 AOV) cannot list genuine leather products on Printify today, forcing them to route premium transactions to PrintKK — despite its 50-unit MOQ. If we fix the taxonomy (MAT-001) and add laser engraving with 1-unit MOQ, they will consolidate their leather spend on Printify, validated at ≥$150K GMV/month within 90 days of launch.</t>
         </is>
@@ -4605,7 +4689,7 @@
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="63" t="inlineStr">
+      <c r="A11" s="65" t="inlineStr">
         <is>
           <t>SOM — Year 2</t>
         </is>
@@ -4637,7 +4721,7 @@
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="64" t="inlineStr">
+      <c r="A12" s="66" t="inlineStr">
         <is>
           <t>SOM — Year 5</t>
         </is>
@@ -4701,12 +4785,12 @@
       </c>
     </row>
     <row r="17" ht="28" customHeight="1">
-      <c r="A17" s="65" t="inlineStr">
+      <c r="A17" s="67" t="inlineStr">
         <is>
           <t>Zero structured-taxonomy player</t>
         </is>
       </c>
-      <c r="B17" s="66" t="inlineStr">
+      <c r="B17" s="68" t="inlineStr">
         <is>
           <t>No POD platform has leather taxonomy + FTC compliance today</t>
         </is>
@@ -4735,12 +4819,12 @@
       </c>
     </row>
     <row r="19" ht="28" customHeight="1">
-      <c r="A19" s="65" t="inlineStr">
+      <c r="A19" s="67" t="inlineStr">
         <is>
           <t>Amazon demand confirmed</t>
         </is>
       </c>
-      <c r="B19" s="66" t="inlineStr">
+      <c r="B19" s="68" t="inlineStr">
         <is>
           <t>BULLIANT wallet: 8,365 units/mo BSR — top POD leather SKU (accio.com 2025)</t>
         </is>
@@ -4769,12 +4853,12 @@
       </c>
     </row>
     <row r="21" ht="28" customHeight="1">
-      <c r="A21" s="65" t="inlineStr">
+      <c r="A21" s="67" t="inlineStr">
         <is>
           <t>PrintKK dependency cost</t>
         </is>
       </c>
-      <c r="B21" s="66" t="inlineStr">
+      <c r="B21" s="68" t="inlineStr">
         <is>
           <t>Decorators using PrintKK: 50-unit MOQ, no FTC compliance, no portal</t>
         </is>
@@ -4811,7 +4895,7 @@
       </c>
     </row>
     <row r="25" ht="180" customHeight="1">
-      <c r="A25" s="67" t="inlineStr">
+      <c r="A25" s="69" t="inlineStr">
         <is>
           <t>THE 5 INITIATIVES WE PROPOSE:
 ① PoC (W0 · $0) — Before writing a single line of code, the PM validates the supply side: outreach to 50 existing Printify Decorators, obtain ≥5 signed LOIs, confirm supplier SLA (1-unit MOQ, laser engraving). If no LOIs → cancel. Cost: zero.
@@ -5096,31 +5180,31 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="68" t="inlineStr">
+      <c r="A36" s="70" t="inlineStr">
         <is>
           <t>Conservative</t>
         </is>
       </c>
-      <c r="B36" s="69" t="n">
+      <c r="B36" s="71" t="n">
         <v>8</v>
       </c>
-      <c r="C36" s="70" t="n">
+      <c r="C36" s="72" t="n">
         <v>60000</v>
       </c>
-      <c r="D36" s="70" t="n">
+      <c r="D36" s="72" t="n">
         <v>720000</v>
       </c>
-      <c r="E36" s="69" t="inlineStr">
+      <c r="E36" s="71" t="inlineStr">
         <is>
           <t>&gt; 36 months</t>
         </is>
       </c>
-      <c r="F36" s="68" t="inlineStr">
+      <c r="F36" s="70" t="inlineStr">
         <is>
           <t>KILL at Month 2 Gate (&lt; 15 orders)</t>
         </is>
       </c>
-      <c r="G36" s="71" t="inlineStr">
+      <c r="G36" s="73" t="inlineStr">
         <is>
           <t>POD industry average — Printify data</t>
         </is>
@@ -5132,16 +5216,16 @@
           <t>Base Case</t>
         </is>
       </c>
-      <c r="B37" s="72" t="n">
+      <c r="B37" s="74" t="n">
         <v>20</v>
       </c>
-      <c r="C37" s="73" t="n">
+      <c r="C37" s="75" t="n">
         <v>150000</v>
       </c>
-      <c r="D37" s="73" t="n">
+      <c r="D37" s="75" t="n">
         <v>1800000</v>
       </c>
-      <c r="E37" s="72" t="inlineStr">
+      <c r="E37" s="74" t="inlineStr">
         <is>
           <t>~15–17 months</t>
         </is>
@@ -5158,7 +5242,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="64" t="inlineStr">
+      <c r="A38" s="66" t="inlineStr">
         <is>
           <t>Optimistic</t>
         </is>
@@ -5166,10 +5250,10 @@
       <c r="B38" s="49" t="n">
         <v>50</v>
       </c>
-      <c r="C38" s="74" t="n">
+      <c r="C38" s="76" t="n">
         <v>375000</v>
       </c>
-      <c r="D38" s="74" t="n">
+      <c r="D38" s="76" t="n">
         <v>4500000</v>
       </c>
       <c r="E38" s="49" t="inlineStr">
@@ -5177,7 +5261,7 @@
           <t>~9–10 months</t>
         </is>
       </c>
-      <c r="F38" s="64" t="inlineStr">
+      <c r="F38" s="66" t="inlineStr">
         <is>
           <t>SCALE to 1,500+ SKUs</t>
         </is>
@@ -5301,32 +5385,32 @@
           <t>Gate 0 · PoC</t>
         </is>
       </c>
-      <c r="B66" s="75" t="inlineStr">
+      <c r="B66" s="77" t="inlineStr">
         <is>
           <t>W0</t>
         </is>
       </c>
-      <c r="C66" s="75" t="inlineStr">
+      <c r="C66" s="77" t="inlineStr">
         <is>
           <t>≥ 5 Signed LOIs + Supplier SLA ready</t>
         </is>
       </c>
-      <c r="D66" s="76" t="inlineStr">
+      <c r="D66" s="78" t="inlineStr">
         <is>
           <t>Approve ~$20K for Design Sprint</t>
         </is>
       </c>
-      <c r="E66" s="77" t="inlineStr">
+      <c r="E66" s="79" t="inlineStr">
         <is>
           <t>CANCEL — $0 engineering spent</t>
         </is>
       </c>
-      <c r="F66" s="75" t="inlineStr">
+      <c r="F66" s="77" t="inlineStr">
         <is>
           <t>$0</t>
         </is>
       </c>
-      <c r="G66" s="75" t="inlineStr">
+      <c r="G66" s="77" t="inlineStr">
         <is>
           <t>Demand signal before any code written</t>
         </is>
@@ -5338,32 +5422,32 @@
           <t>Gate 1 · MVP 2</t>
         </is>
       </c>
-      <c r="B67" s="78" t="inlineStr">
+      <c r="B67" s="80" t="inlineStr">
         <is>
           <t>W16</t>
         </is>
       </c>
-      <c r="C67" s="78" t="inlineStr">
+      <c r="C67" s="80" t="inlineStr">
         <is>
           <t>150 valid SKUs; portal error &lt; 10%</t>
         </is>
       </c>
-      <c r="D67" s="79" t="inlineStr">
+      <c r="D67" s="81" t="inlineStr">
         <is>
           <t>Proceed to Marketplace Integrations</t>
         </is>
       </c>
-      <c r="E67" s="80" t="inlineStr">
+      <c r="E67" s="82" t="inlineStr">
         <is>
           <t>PAUSE — redesign portal UI &amp; AI flow</t>
         </is>
       </c>
-      <c r="F67" s="78" t="inlineStr">
+      <c r="F67" s="80" t="inlineStr">
         <is>
           <t>~$220K</t>
         </is>
       </c>
-      <c r="G67" s="78" t="inlineStr">
+      <c r="G67" s="80" t="inlineStr">
         <is>
           <t>Supply readiness before marketplace spend</t>
         </is>
@@ -5375,32 +5459,32 @@
           <t>Gate 2 · M2</t>
         </is>
       </c>
-      <c r="B68" s="81" t="inlineStr">
+      <c r="B68" s="83" t="inlineStr">
         <is>
           <t>Month 2</t>
         </is>
       </c>
-      <c r="C68" s="81" t="inlineStr">
+      <c r="C68" s="83" t="inlineStr">
         <is>
           <t>≥ 20 orders / SKU / month</t>
         </is>
       </c>
-      <c r="D68" s="82" t="inlineStr">
+      <c r="D68" s="84" t="inlineStr">
         <is>
           <t>FULL SCALE — expand to 1,500+ SKUs</t>
         </is>
       </c>
-      <c r="E68" s="83" t="inlineStr">
+      <c r="E68" s="85" t="inlineStr">
         <is>
           <t>KILL (&lt; 15) — halt &amp; reallocate team</t>
         </is>
       </c>
-      <c r="F68" s="81" t="inlineStr">
+      <c r="F68" s="83" t="inlineStr">
         <is>
           <t>~$340K</t>
         </is>
       </c>
-      <c r="G68" s="81" t="inlineStr">
+      <c r="G68" s="83" t="inlineStr">
         <is>
           <t>M1 has launch noise; M2 = true organic signal</t>
         </is>
@@ -5412,22 +5496,22 @@
           <t>M9</t>
         </is>
       </c>
-      <c r="B69" s="84" t="n">
+      <c r="B69" s="86" t="n">
         <v>55</v>
       </c>
-      <c r="C69" s="85" t="n">
+      <c r="C69" s="87" t="n">
         <v>130</v>
       </c>
-      <c r="D69" s="86" t="n">
+      <c r="D69" s="88" t="n">
         <v>320</v>
       </c>
-      <c r="E69" s="87" t="n">
+      <c r="E69" s="89" t="n">
         <v>60</v>
       </c>
-      <c r="F69" s="88" t="n">
+      <c r="F69" s="90" t="n">
         <v>150</v>
       </c>
-      <c r="G69" s="89" t="n">
+      <c r="G69" s="91" t="n">
         <v>375</v>
       </c>
     </row>
@@ -5437,22 +5521,22 @@
           <t>M12</t>
         </is>
       </c>
-      <c r="B70" s="90" t="n">
+      <c r="B70" s="92" t="n">
         <v>60</v>
       </c>
-      <c r="C70" s="91" t="n">
+      <c r="C70" s="93" t="n">
         <v>150</v>
       </c>
-      <c r="D70" s="92" t="n">
+      <c r="D70" s="94" t="n">
         <v>375</v>
       </c>
-      <c r="E70" s="87" t="n">
+      <c r="E70" s="89" t="n">
         <v>60</v>
       </c>
-      <c r="F70" s="88" t="n">
+      <c r="F70" s="90" t="n">
         <v>150</v>
       </c>
-      <c r="G70" s="89" t="n">
+      <c r="G70" s="91" t="n">
         <v>375</v>
       </c>
     </row>
@@ -5501,12 +5585,12 @@
           <t>Decorators</t>
         </is>
       </c>
-      <c r="B73" s="93" t="inlineStr">
+      <c r="B73" s="95" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="C73" s="94" t="inlineStr">
+      <c r="C73" s="96" t="inlineStr">
         <is>
           <t>20</t>
         </is>
@@ -5533,12 +5617,12 @@
           <t>Orders/SKU/month</t>
         </is>
       </c>
-      <c r="B74" s="95" t="inlineStr">
+      <c r="B74" s="97" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="C74" s="94" t="inlineStr">
+      <c r="C74" s="96" t="inlineStr">
         <is>
           <t>20</t>
         </is>
@@ -5565,12 +5649,12 @@
           <t>Monthly margin</t>
         </is>
       </c>
-      <c r="B75" s="93" t="inlineStr">
+      <c r="B75" s="95" t="inlineStr">
         <is>
           <t>$60K</t>
         </is>
       </c>
-      <c r="C75" s="94" t="inlineStr">
+      <c r="C75" s="96" t="inlineStr">
         <is>
           <t>$150K</t>
         </is>
@@ -5597,12 +5681,12 @@
           <t>Annual run-rate</t>
         </is>
       </c>
-      <c r="B76" s="95" t="inlineStr">
+      <c r="B76" s="97" t="inlineStr">
         <is>
           <t>$720K</t>
         </is>
       </c>
-      <c r="C76" s="94" t="inlineStr">
+      <c r="C76" s="96" t="inlineStr">
         <is>
           <t>$1.8M</t>
         </is>
@@ -5629,12 +5713,12 @@
           <t>Payback period</t>
         </is>
       </c>
-      <c r="B77" s="93" t="inlineStr">
+      <c r="B77" s="95" t="inlineStr">
         <is>
           <t>&gt; 36 mo</t>
         </is>
       </c>
-      <c r="C77" s="94" t="inlineStr">
+      <c r="C77" s="96" t="inlineStr">
         <is>
           <t>~16 mo</t>
         </is>
@@ -5661,12 +5745,12 @@
           <t>Total investment</t>
         </is>
       </c>
-      <c r="B78" s="95" t="inlineStr">
+      <c r="B78" s="97" t="inlineStr">
         <is>
           <t>$340K</t>
         </is>
       </c>
-      <c r="C78" s="94" t="inlineStr">
+      <c r="C78" s="96" t="inlineStr">
         <is>
           <t>$340K</t>
         </is>
@@ -5693,27 +5777,27 @@
           <t>Decision at M2</t>
         </is>
       </c>
-      <c r="B79" s="69" t="inlineStr">
+      <c r="B79" s="71" t="inlineStr">
         <is>
           <t>KILL</t>
         </is>
       </c>
-      <c r="C79" s="94" t="inlineStr">
+      <c r="C79" s="96" t="inlineStr">
         <is>
           <t>GO</t>
         </is>
       </c>
-      <c r="D79" s="96" t="inlineStr">
+      <c r="D79" s="98" t="inlineStr">
         <is>
           <t>SCALE</t>
         </is>
       </c>
-      <c r="E79" s="97" t="inlineStr">
+      <c r="E79" s="99" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F79" s="97" t="inlineStr">
+      <c r="F79" s="99" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -5830,37 +5914,37 @@
           <t>Genuine leather products (Full-Grain / Top-Grain)</t>
         </is>
       </c>
-      <c r="B5" s="93" t="inlineStr">
+      <c r="B5" s="95" t="inlineStr">
         <is>
           <t>❌ 0</t>
         </is>
       </c>
-      <c r="C5" s="98" t="inlineStr">
+      <c r="C5" s="100" t="inlineStr">
         <is>
           <t>✅ 150+ SKUs</t>
         </is>
       </c>
-      <c r="D5" s="93" t="inlineStr">
+      <c r="D5" s="95" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="E5" s="93" t="inlineStr">
+      <c r="E5" s="95" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="F5" s="93" t="inlineStr">
+      <c r="F5" s="95" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="G5" s="93" t="inlineStr">
+      <c r="G5" s="95" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="H5" s="93" t="inlineStr">
+      <c r="H5" s="95" t="inlineStr">
         <is>
           <t>⚠ Yes, no standards</t>
         </is>
@@ -5877,7 +5961,7 @@
           <t>✅ ~45</t>
         </is>
       </c>
-      <c r="C6" s="98" t="inlineStr">
+      <c r="C6" s="100" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -5914,37 +5998,37 @@
           <t>Material taxonomy (tier classification)</t>
         </is>
       </c>
-      <c r="B7" s="93" t="inlineStr">
+      <c r="B7" s="95" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="C7" s="98" t="inlineStr">
+      <c r="C7" s="100" t="inlineStr">
         <is>
           <t>✅ 8 fields</t>
         </is>
       </c>
-      <c r="D7" s="93" t="inlineStr">
+      <c r="D7" s="95" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="E7" s="93" t="inlineStr">
+      <c r="E7" s="95" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="F7" s="93" t="inlineStr">
+      <c r="F7" s="95" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="G7" s="93" t="inlineStr">
+      <c r="G7" s="95" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="H7" s="93" t="inlineStr">
+      <c r="H7" s="95" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
@@ -5956,37 +6040,37 @@
           <t>FTC compliance / auto-reject mislabeling</t>
         </is>
       </c>
-      <c r="B8" s="95" t="inlineStr">
+      <c r="B8" s="97" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="C8" s="98" t="inlineStr">
+      <c r="C8" s="100" t="inlineStr">
         <is>
           <t>✅ MAT-001</t>
         </is>
       </c>
-      <c r="D8" s="95" t="inlineStr">
+      <c r="D8" s="97" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="E8" s="95" t="inlineStr">
+      <c r="E8" s="97" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="F8" s="95" t="inlineStr">
+      <c r="F8" s="97" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="G8" s="95" t="inlineStr">
+      <c r="G8" s="97" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="H8" s="95" t="inlineStr">
+      <c r="H8" s="97" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
@@ -5998,32 +6082,32 @@
           <t>Laser engraving support</t>
         </is>
       </c>
-      <c r="B9" s="93" t="inlineStr">
+      <c r="B9" s="95" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="C9" s="98" t="inlineStr">
+      <c r="C9" s="100" t="inlineStr">
         <is>
           <t>✅ MVP 1</t>
         </is>
       </c>
-      <c r="D9" s="93" t="inlineStr">
+      <c r="D9" s="95" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="E9" s="93" t="inlineStr">
+      <c r="E9" s="95" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="F9" s="93" t="inlineStr">
+      <c r="F9" s="95" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="G9" s="93" t="inlineStr">
+      <c r="G9" s="95" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
@@ -6040,37 +6124,37 @@
           <t>Debossing support</t>
         </is>
       </c>
-      <c r="B10" s="95" t="inlineStr">
+      <c r="B10" s="97" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="C10" s="98" t="inlineStr">
+      <c r="C10" s="100" t="inlineStr">
         <is>
           <t>✅ MVP 1</t>
         </is>
       </c>
-      <c r="D10" s="95" t="inlineStr">
+      <c r="D10" s="97" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="E10" s="95" t="inlineStr">
+      <c r="E10" s="97" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="F10" s="95" t="inlineStr">
+      <c r="F10" s="97" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="G10" s="95" t="inlineStr">
+      <c r="G10" s="97" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="H10" s="95" t="inlineStr">
+      <c r="H10" s="97" t="inlineStr">
         <is>
           <t>⚠ Partial</t>
         </is>
@@ -6082,12 +6166,12 @@
           <t>Leather mockup engine</t>
         </is>
       </c>
-      <c r="B11" s="93" t="inlineStr">
+      <c r="B11" s="95" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="C11" s="98" t="inlineStr">
+      <c r="C11" s="100" t="inlineStr">
         <is>
           <t>✅ MVP 2</t>
         </is>
@@ -6097,22 +6181,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E11" s="93" t="inlineStr">
+      <c r="E11" s="95" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="F11" s="93" t="inlineStr">
+      <c r="F11" s="95" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="G11" s="93" t="inlineStr">
+      <c r="G11" s="95" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="H11" s="93" t="inlineStr">
+      <c r="H11" s="95" t="inlineStr">
         <is>
           <t>⚠ Basic</t>
         </is>
@@ -6124,37 +6208,37 @@
           <t>Decorator self-onboard portal (leather)</t>
         </is>
       </c>
-      <c r="B12" s="95" t="inlineStr">
+      <c r="B12" s="97" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="C12" s="98" t="inlineStr">
+      <c r="C12" s="100" t="inlineStr">
         <is>
           <t>✅ MVP 2</t>
         </is>
       </c>
-      <c r="D12" s="95" t="inlineStr">
+      <c r="D12" s="97" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="E12" s="95" t="inlineStr">
+      <c r="E12" s="97" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="F12" s="95" t="inlineStr">
+      <c r="F12" s="97" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="G12" s="95" t="inlineStr">
+      <c r="G12" s="97" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="H12" s="95" t="inlineStr">
+      <c r="H12" s="97" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
@@ -6166,37 +6250,37 @@
           <t>AI field-assist for material attributes</t>
         </is>
       </c>
-      <c r="B13" s="93" t="inlineStr">
+      <c r="B13" s="95" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="C13" s="98" t="inlineStr">
+      <c r="C13" s="100" t="inlineStr">
         <is>
           <t>✅ MVP 2</t>
         </is>
       </c>
-      <c r="D13" s="93" t="inlineStr">
+      <c r="D13" s="95" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="E13" s="93" t="inlineStr">
+      <c r="E13" s="95" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="F13" s="93" t="inlineStr">
+      <c r="F13" s="95" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="G13" s="93" t="inlineStr">
+      <c r="G13" s="95" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="H13" s="93" t="inlineStr">
+      <c r="H13" s="95" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
@@ -6208,37 +6292,37 @@
           <t>Prop 65 auto-disclosure (CA / Amazon)</t>
         </is>
       </c>
-      <c r="B14" s="95" t="inlineStr">
+      <c r="B14" s="97" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="C14" s="98" t="inlineStr">
+      <c r="C14" s="100" t="inlineStr">
         <is>
           <t>✅ MVP 3</t>
         </is>
       </c>
-      <c r="D14" s="95" t="inlineStr">
+      <c r="D14" s="97" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="E14" s="95" t="inlineStr">
+      <c r="E14" s="97" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="F14" s="95" t="inlineStr">
+      <c r="F14" s="97" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="G14" s="95" t="inlineStr">
+      <c r="G14" s="97" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="H14" s="95" t="inlineStr">
+      <c r="H14" s="97" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
@@ -6250,12 +6334,12 @@
           <t>Amazon SP-API leather category</t>
         </is>
       </c>
-      <c r="B15" s="93" t="inlineStr">
+      <c r="B15" s="95" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="C15" s="98" t="inlineStr">
+      <c r="C15" s="100" t="inlineStr">
         <is>
           <t>✅ MVP 3</t>
         </is>
@@ -6265,22 +6349,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E15" s="93" t="inlineStr">
+      <c r="E15" s="95" t="inlineStr">
         <is>
           <t>⚠</t>
         </is>
       </c>
-      <c r="F15" s="93" t="inlineStr">
+      <c r="F15" s="95" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="G15" s="93" t="inlineStr">
+      <c r="G15" s="95" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="H15" s="93" t="inlineStr">
+      <c r="H15" s="95" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
@@ -6292,37 +6376,37 @@
           <t>LWG / Oeko-Tex certification field</t>
         </is>
       </c>
-      <c r="B16" s="95" t="inlineStr">
+      <c r="B16" s="97" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="C16" s="99" t="inlineStr">
+      <c r="C16" s="101" t="inlineStr">
         <is>
           <t>⏳ V2</t>
         </is>
       </c>
-      <c r="D16" s="95" t="inlineStr">
+      <c r="D16" s="97" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="E16" s="95" t="inlineStr">
+      <c r="E16" s="97" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="F16" s="95" t="inlineStr">
+      <c r="F16" s="97" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="G16" s="95" t="inlineStr">
+      <c r="G16" s="97" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="H16" s="95" t="inlineStr">
+      <c r="H16" s="97" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
@@ -6334,12 +6418,12 @@
           <t>Etsy material attribute mapping</t>
         </is>
       </c>
-      <c r="B17" s="93" t="inlineStr">
+      <c r="B17" s="95" t="inlineStr">
         <is>
           <t>⚠ Generic</t>
         </is>
       </c>
-      <c r="C17" s="98" t="inlineStr">
+      <c r="C17" s="100" t="inlineStr">
         <is>
           <t>✅ MVP 3</t>
         </is>
@@ -6354,17 +6438,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F17" s="93" t="inlineStr">
+      <c r="F17" s="95" t="inlineStr">
         <is>
           <t>⚠</t>
         </is>
       </c>
-      <c r="G17" s="93" t="inlineStr">
+      <c r="G17" s="95" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="H17" s="93" t="inlineStr">
+      <c r="H17" s="95" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
@@ -6571,7 +6655,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="65" t="inlineStr">
+      <c r="A27" s="67" t="inlineStr">
         <is>
           <t>Printify</t>
         </is>
@@ -6891,196 +6975,196 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="100" t="inlineStr">
+      <c r="A13" s="102" t="inlineStr">
         <is>
           <t>Phase</t>
         </is>
       </c>
-      <c r="B13" s="101" t="inlineStr">
+      <c r="B13" s="103" t="inlineStr">
         <is>
           <t>W0</t>
         </is>
       </c>
-      <c r="C13" s="101" t="inlineStr">
+      <c r="C13" s="103" t="inlineStr">
         <is>
           <t>W1</t>
         </is>
       </c>
-      <c r="D13" s="101" t="inlineStr">
+      <c r="D13" s="103" t="inlineStr">
         <is>
           <t>W2</t>
         </is>
       </c>
-      <c r="E13" s="101" t="inlineStr">
+      <c r="E13" s="103" t="inlineStr">
         <is>
           <t>W3</t>
         </is>
       </c>
-      <c r="F13" s="101" t="inlineStr">
+      <c r="F13" s="103" t="inlineStr">
         <is>
           <t>W4</t>
         </is>
       </c>
-      <c r="G13" s="101" t="inlineStr">
+      <c r="G13" s="103" t="inlineStr">
         <is>
           <t>W5</t>
         </is>
       </c>
-      <c r="H13" s="101" t="inlineStr">
+      <c r="H13" s="103" t="inlineStr">
         <is>
           <t>W6</t>
         </is>
       </c>
-      <c r="I13" s="101" t="inlineStr">
+      <c r="I13" s="103" t="inlineStr">
         <is>
           <t>W7</t>
         </is>
       </c>
-      <c r="J13" s="101" t="inlineStr">
+      <c r="J13" s="103" t="inlineStr">
         <is>
           <t>W8</t>
         </is>
       </c>
-      <c r="K13" s="101" t="inlineStr">
+      <c r="K13" s="103" t="inlineStr">
         <is>
           <t>W9</t>
         </is>
       </c>
-      <c r="L13" s="101" t="inlineStr">
+      <c r="L13" s="103" t="inlineStr">
         <is>
           <t>W10</t>
         </is>
       </c>
-      <c r="M13" s="101" t="inlineStr">
+      <c r="M13" s="103" t="inlineStr">
         <is>
           <t>W11</t>
         </is>
       </c>
-      <c r="N13" s="101" t="inlineStr">
+      <c r="N13" s="103" t="inlineStr">
         <is>
           <t>W12</t>
         </is>
       </c>
-      <c r="O13" s="101" t="inlineStr">
+      <c r="O13" s="103" t="inlineStr">
         <is>
           <t>W13</t>
         </is>
       </c>
-      <c r="P13" s="101" t="inlineStr">
+      <c r="P13" s="103" t="inlineStr">
         <is>
           <t>W14</t>
         </is>
       </c>
-      <c r="Q13" s="101" t="inlineStr">
+      <c r="Q13" s="103" t="inlineStr">
         <is>
           <t>W15</t>
         </is>
       </c>
-      <c r="R13" s="101" t="inlineStr">
+      <c r="R13" s="103" t="inlineStr">
         <is>
           <t>W16</t>
         </is>
       </c>
-      <c r="S13" s="101" t="inlineStr">
+      <c r="S13" s="103" t="inlineStr">
         <is>
           <t>W17</t>
         </is>
       </c>
-      <c r="T13" s="101" t="inlineStr">
+      <c r="T13" s="103" t="inlineStr">
         <is>
           <t>W18</t>
         </is>
       </c>
-      <c r="U13" s="101" t="inlineStr">
+      <c r="U13" s="103" t="inlineStr">
         <is>
           <t>W19</t>
         </is>
       </c>
-      <c r="V13" s="101" t="inlineStr">
+      <c r="V13" s="103" t="inlineStr">
         <is>
           <t>W20</t>
         </is>
       </c>
-      <c r="W13" s="101" t="inlineStr">
+      <c r="W13" s="103" t="inlineStr">
         <is>
           <t>W21</t>
         </is>
       </c>
-      <c r="X13" s="101" t="inlineStr">
+      <c r="X13" s="103" t="inlineStr">
         <is>
           <t>W22</t>
         </is>
       </c>
-      <c r="Y13" s="101" t="inlineStr">
+      <c r="Y13" s="103" t="inlineStr">
         <is>
           <t>W23</t>
         </is>
       </c>
-      <c r="Z13" s="101" t="inlineStr">
+      <c r="Z13" s="103" t="inlineStr">
         <is>
           <t>W24</t>
         </is>
       </c>
     </row>
     <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="102" t="inlineStr">
+      <c r="A14" s="104" t="inlineStr">
         <is>
           <t>PoC</t>
         </is>
       </c>
-      <c r="B14" s="103" t="n"/>
+      <c r="B14" s="105" t="n"/>
     </row>
     <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="102" t="inlineStr">
+      <c r="A15" s="104" t="inlineStr">
         <is>
           <t>Design Sprint</t>
         </is>
       </c>
-      <c r="C15" s="104" t="n"/>
-      <c r="D15" s="104" t="n"/>
+      <c r="C15" s="106" t="n"/>
+      <c r="D15" s="106" t="n"/>
     </row>
     <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="102" t="inlineStr">
+      <c r="A16" s="104" t="inlineStr">
         <is>
           <t>MVP 1 — Schema</t>
         </is>
       </c>
-      <c r="E16" s="105" t="n"/>
-      <c r="F16" s="105" t="n"/>
-      <c r="G16" s="105" t="n"/>
-      <c r="H16" s="105" t="n"/>
-      <c r="I16" s="105" t="n"/>
-      <c r="J16" s="105" t="n"/>
+      <c r="E16" s="107" t="n"/>
+      <c r="F16" s="107" t="n"/>
+      <c r="G16" s="107" t="n"/>
+      <c r="H16" s="107" t="n"/>
+      <c r="I16" s="107" t="n"/>
+      <c r="J16" s="107" t="n"/>
     </row>
     <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="102" t="inlineStr">
+      <c r="A17" s="104" t="inlineStr">
         <is>
           <t>MVP 2 — Mockup</t>
         </is>
       </c>
-      <c r="K17" s="106" t="n"/>
-      <c r="L17" s="106" t="n"/>
-      <c r="M17" s="106" t="n"/>
-      <c r="N17" s="106" t="n"/>
-      <c r="O17" s="106" t="n"/>
-      <c r="P17" s="106" t="n"/>
-      <c r="Q17" s="106" t="n"/>
-      <c r="R17" s="106" t="n"/>
+      <c r="K17" s="108" t="n"/>
+      <c r="L17" s="108" t="n"/>
+      <c r="M17" s="108" t="n"/>
+      <c r="N17" s="108" t="n"/>
+      <c r="O17" s="108" t="n"/>
+      <c r="P17" s="108" t="n"/>
+      <c r="Q17" s="108" t="n"/>
+      <c r="R17" s="108" t="n"/>
     </row>
     <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="102" t="inlineStr">
+      <c r="A18" s="104" t="inlineStr">
         <is>
           <t>MVP 3 — Channels</t>
         </is>
       </c>
-      <c r="S18" s="107" t="n"/>
-      <c r="T18" s="107" t="n"/>
-      <c r="U18" s="107" t="n"/>
-      <c r="V18" s="107" t="n"/>
-      <c r="W18" s="107" t="n"/>
-      <c r="X18" s="107" t="n"/>
-      <c r="Y18" s="107" t="n"/>
-      <c r="Z18" s="107" t="n"/>
+      <c r="S18" s="109" t="n"/>
+      <c r="T18" s="109" t="n"/>
+      <c r="U18" s="109" t="n"/>
+      <c r="V18" s="109" t="n"/>
+      <c r="W18" s="109" t="n"/>
+      <c r="X18" s="109" t="n"/>
+      <c r="Y18" s="109" t="n"/>
+      <c r="Z18" s="109" t="n"/>
     </row>
     <row r="21" customHeight="1">
       <c r="A21" t="inlineStr">
@@ -7716,7 +7800,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="108" t="inlineStr">
+      <c r="A12" s="110" t="inlineStr">
         <is>
           <t>lwg_grade</t>
         </is>
@@ -7748,7 +7832,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="109" t="inlineStr">
+      <c r="A13" s="111" t="inlineStr">
         <is>
           <t>oeko_tex_cert_id</t>
         </is>
@@ -7776,7 +7860,7 @@
       <c r="F13" s="51" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="108" t="inlineStr">
+      <c r="A14" s="110" t="inlineStr">
         <is>
           <t>reach_cr_vi_compliant</t>
         </is>
@@ -8064,7 +8148,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="109" t="inlineStr">
+      <c r="A29" s="111" t="inlineStr">
         <is>
           <t>TikTok Shop</t>
         </is>
@@ -8092,7 +8176,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="108" t="inlineStr">
+      <c r="A30" s="110" t="inlineStr">
         <is>
           <t>PrestaShop</t>
         </is>

</xml_diff>

<commit_message>
Excel: fix field count to 8 everywhere — consistent with PRD
- Implementation Map: replace 10-field table (7 old MVP1 + 3 V2) with 8 PRD fields
  leather_grade, tanning_method, finish_type, hide_thickness_mm, hide_origin,
  grain_correction, compliance_cert (MVP1) + eco_claims (MVP2)
- Business Case intro: "7 new blueprint API fields" → "8 new blueprint schema fields"
- Section header: "(10 new fields)" → "(8 new fields)"

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/Printify_Leather_PRD_Workbook.xlsx
+++ b/output/Printify_Leather_PRD_Workbook.xlsx
@@ -604,10 +604,10 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -4900,7 +4900,7 @@
           <t>THE 5 INITIATIVES WE PROPOSE:
 ① PoC (W0 · $0) — Before writing a single line of code, the PM validates the supply side: outreach to 50 existing Printify Decorators, obtain ≥5 signed LOIs, confirm supplier SLA (1-unit MOQ, laser engraving). If no LOIs → cancel. Cost: zero.
 ② Design Sprint (W1–2 · $20K) — UX designs the Decorator portal and the MAT-001 scoring state UI. Plain-language field labels replace technical jargon. New DS components (quality tier indicator, ECO badge, compliance banner) are built once and reused across all surfaces.
-③ MVP 1 — Schema &amp; Classifier (W3–8 · $80K) — Engineers add 7 new blueprint API fields (material_tier, tannage_method, origin_country, finish_type, thickness_mm, prop_65_compliant, laser_engraving_area). The MAT-001 LLM classifier auto-rejects PU/bonded leather mislabeled as "genuine". Kill gate: ≥88% auto-approval, &lt;2% false positives.
+③ MVP 1 — Schema &amp; Classifier (W3–8 · $80K) — Engineers add 8 new blueprint schema fields (leather_grade, tanning_method, finish_type, hide_thickness_mm, hide_origin, grain_correction, compliance_cert, eco_claims). The MAT-001 LLM classifier auto-rejects PU/bonded leather mislabeled as "genuine". Kill gate: ≥88% auto-approval, &lt;2% false positives.
 ④ MVP 2 — Mockup Engine + Shopify Pilot (W9–16 · $120K) — Static leather texture mockup engine (3 textures/tier). AI field-assist agent pre-fills schema fields from supplier data. 5 pilot Decorators onboard and create 150 approved SKUs. Shopify metafield integration ★ goes live at W12 — immediate demand signal before Etsy/Amazon launch.
 ⑤ MVP 3 — Marketplace Launch (W17–24 · $120K) — 150 SKUs go live across Etsy, Amazon (SP-API, Prop 65), and WooCommerce. Month 1 demand read. Kill decision at Month 2: &lt;15 orders/SKU → halt &amp; reallocate; ≥20 → full scale to 1,500+ SKUs.</t>
         </is>
@@ -7529,7 +7529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -7551,7 +7551,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>1. Blueprint API Schema Extensions (10 new fields)</t>
+          <t>1. Blueprint API Schema Extensions (8 new fields)</t>
         </is>
       </c>
     </row>
@@ -7590,7 +7590,7 @@
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>material_tier</t>
+          <t>leather_grade</t>
         </is>
       </c>
       <c r="B5" s="10" t="inlineStr">
@@ -7600,7 +7600,7 @@
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>full_grain / top_grain / split / bonded / pu / vegan</t>
+          <t>full_grain / top_grain / corrected_grain / split / bonded / pu / vegan</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
@@ -7610,7 +7610,7 @@
       </c>
       <c r="E5" s="10" t="inlineStr">
         <is>
-          <t>Etsy: material attr · Amazon: LeatherType node · Shopify: metafield</t>
+          <t>Etsy: material attr · Amazon: LeatherType node · Shopify: metafield · FTC MAT-001 anchor</t>
         </is>
       </c>
       <c r="F5" s="54" t="inlineStr">
@@ -7622,7 +7622,7 @@
     <row r="6">
       <c r="A6" s="33" t="inlineStr">
         <is>
-          <t>tannage_method</t>
+          <t>tanning_method</t>
         </is>
       </c>
       <c r="B6" s="18" t="inlineStr">
@@ -7632,7 +7632,7 @@
       </c>
       <c r="C6" s="18" t="inlineStr">
         <is>
-          <t>vegetable / chrome / combination</t>
+          <t>vegetable / chrome / chrome_free / combination</t>
         </is>
       </c>
       <c r="D6" s="18" t="inlineStr">
@@ -7654,17 +7654,17 @@
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>origin_country</t>
+          <t>finish_type</t>
         </is>
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>ISO 3166</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>e.g. IT, US, MX</t>
+          <t>smooth / pebbled / suede / patent / nubuck</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
@@ -7674,7 +7674,7 @@
       </c>
       <c r="E7" s="10" t="inlineStr">
         <is>
-          <t>Amazon origin attribute · Etsy origin filter</t>
+          <t>Mockup engine texture selector · Etsy search filter</t>
         </is>
       </c>
       <c r="F7" s="10" t="inlineStr"/>
@@ -7682,17 +7682,17 @@
     <row r="8">
       <c r="A8" s="33" t="inlineStr">
         <is>
-          <t>finish_type</t>
+          <t>hide_thickness_mm</t>
         </is>
       </c>
       <c r="B8" s="18" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>float</t>
         </is>
       </c>
       <c r="C8" s="18" t="inlineStr">
         <is>
-          <t>smooth / pebbled / suede / patent</t>
+          <t>≥ 0.8mm wallets · ≥ 1.2mm bags · ≥ 2.0mm belts</t>
         </is>
       </c>
       <c r="D8" s="18" t="inlineStr">
@@ -7702,7 +7702,7 @@
       </c>
       <c r="E8" s="18" t="inlineStr">
         <is>
-          <t>Mockup engine texture selector</t>
+          <t>Quality tier display on PDP · pricing premium signal</t>
         </is>
       </c>
       <c r="F8" s="18" t="inlineStr"/>
@@ -7710,17 +7710,17 @@
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>thickness_mm</t>
+          <t>hide_origin</t>
         </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>ISO 3166</t>
         </is>
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>≥ 0.8mm wallets · ≥ 1.2mm bags · ≥ 2.0mm belts</t>
+          <t>e.g. IT, US, MX, IN</t>
         </is>
       </c>
       <c r="D9" s="10" t="inlineStr">
@@ -7730,7 +7730,7 @@
       </c>
       <c r="E9" s="10" t="inlineStr">
         <is>
-          <t>Quality tier display on PDP</t>
+          <t>Amazon origin attribute · Etsy origin filter · premium pricing signal</t>
         </is>
       </c>
       <c r="F9" s="10" t="inlineStr"/>
@@ -7738,7 +7738,7 @@
     <row r="10">
       <c r="A10" s="33" t="inlineStr">
         <is>
-          <t>prop_65_compliant</t>
+          <t>grain_correction</t>
         </is>
       </c>
       <c r="B10" s="18" t="inlineStr">
@@ -7748,7 +7748,7 @@
       </c>
       <c r="C10" s="18" t="inlineStr">
         <is>
-          <t>true / false — required for CA sales &amp; Amazon USA</t>
+          <t>true / false — corrected (sanded) vs. natural grain surface</t>
         </is>
       </c>
       <c r="D10" s="18" t="inlineStr">
@@ -7758,29 +7758,29 @@
       </c>
       <c r="E10" s="18" t="inlineStr">
         <is>
-          <t>Amazon: Prop 65 disclosure auto-populated via SP-API</t>
+          <t>Grade disambiguation: top_grain corrected vs. full_grain natural</t>
         </is>
       </c>
       <c r="F10" s="52" t="inlineStr">
         <is>
-          <t>false = block listing on Amazon channel</t>
+          <t>Required to prevent misclassification at ingestion</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>laser_engraving_area</t>
+          <t>compliance_cert</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>object</t>
+          <t>enum[]</t>
         </is>
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>{width_mm: float, height_mm: float}</t>
+          <t>ftc_genuine / prop_65_ca / mat_001_approved / none</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
@@ -7790,270 +7790,274 @@
       </c>
       <c r="E11" s="10" t="inlineStr">
         <is>
-          <t>Decoration method selector + mockup overlay</t>
+          <t>Amazon: Prop 65 auto-disclosure · MAT-001 classifier output · listing gate</t>
         </is>
       </c>
       <c r="F11" s="54" t="inlineStr">
         <is>
-          <t>API enum: add laser_engraving + debossing</t>
+          <t>none = block on Amazon channel</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="110" t="inlineStr">
-        <is>
-          <t>lwg_grade</t>
-        </is>
-      </c>
-      <c r="B12" s="47" t="inlineStr">
-        <is>
-          <t>enum</t>
-        </is>
-      </c>
-      <c r="C12" s="47" t="inlineStr">
-        <is>
-          <t>gold / silver / bronze</t>
-        </is>
-      </c>
-      <c r="D12" s="47" t="inlineStr">
-        <is>
-          <t>V2</t>
-        </is>
-      </c>
-      <c r="E12" s="47" t="inlineStr">
-        <is>
-          <t>ECO badge on PDP · sustainability filter</t>
-        </is>
-      </c>
-      <c r="F12" s="47" t="inlineStr">
-        <is>
-          <t>Requires supplier LWG cert verification</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="111" t="inlineStr">
-        <is>
-          <t>oeko_tex_cert_id</t>
-        </is>
-      </c>
-      <c r="B13" s="51" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="C13" s="51" t="inlineStr">
-        <is>
-          <t>Certificate ID or null</t>
-        </is>
-      </c>
-      <c r="D13" s="51" t="inlineStr">
-        <is>
-          <t>V2</t>
-        </is>
-      </c>
-      <c r="E13" s="51" t="inlineStr">
-        <is>
-          <t>ECO badge · compliance export</t>
-        </is>
-      </c>
-      <c r="F13" s="51" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="110" t="inlineStr">
-        <is>
-          <t>reach_cr_vi_compliant</t>
-        </is>
-      </c>
-      <c r="B14" s="47" t="inlineStr">
-        <is>
-          <t>boolean</t>
-        </is>
-      </c>
-      <c r="C14" s="47" t="inlineStr">
-        <is>
-          <t>Chrome-tanned leather only</t>
-        </is>
-      </c>
-      <c r="D14" s="47" t="inlineStr">
-        <is>
-          <t>V2</t>
-        </is>
-      </c>
-      <c r="E14" s="47" t="inlineStr">
-        <is>
-          <t>EU channel compliance</t>
-        </is>
-      </c>
-      <c r="F14" s="47" t="inlineStr"/>
-    </row>
-    <row r="16" ht="5" customHeight="1"/>
-    <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A12" s="33" t="inlineStr">
+        <is>
+          <t>eco_claims</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>enum[]</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>lwg_gold / lwg_silver / oeko_tex / reach_compliant / none</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>MVP 2</t>
+        </is>
+      </c>
+      <c r="E12" s="18" t="inlineStr">
+        <is>
+          <t>ECO badge on PDP · sustainability filter · EU channel compliance</t>
+        </is>
+      </c>
+      <c r="F12" s="52" t="inlineStr">
+        <is>
+          <t>Requires supplier cert verification</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="5" customHeight="1"/>
+    <row r="15" ht="16" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>2. Native AI Agents</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="28" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Agent</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>MVP</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>Trigger</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>What it does</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>Success metric</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>Failure mode</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="56" customHeight="1">
-      <c r="A19" s="9" t="inlineStr">
+    <row r="17" ht="56" customHeight="1">
+      <c r="A17" s="9" t="inlineStr">
         <is>
           <t>MAT-001 FTC Classifier</t>
         </is>
       </c>
-      <c r="B19" s="10" t="inlineStr">
+      <c r="B17" s="10" t="inlineStr">
         <is>
           <t>MVP 1</t>
         </is>
       </c>
-      <c r="C19" s="10" t="inlineStr">
+      <c r="C17" s="10" t="inlineStr">
         <is>
           <t>Blueprint ingestion — fires on every new leather listing submission</t>
         </is>
       </c>
-      <c r="D19" s="10" t="inlineStr">
+      <c r="D17" s="10" t="inlineStr">
         <is>
           <t>LLM evaluates listing title + material_tier + description. Detects PU/Bonded labeled "Genuine Leather". Auto-rejects non-compliant with corrected label requirement. Zero ops intervention.</t>
         </is>
       </c>
-      <c r="E19" s="10" t="inlineStr">
+      <c r="E17" s="10" t="inlineStr">
         <is>
           <t>Auto-approve ≥ 88% · FP rate &lt; 2%</t>
         </is>
       </c>
-      <c r="F19" s="54" t="inlineStr">
+      <c r="F17" s="54" t="inlineStr">
         <is>
           <t>FP &gt; 2%: legitimate Decorators blocked → churn · FN: PU reaches catalog → FTC risk</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="56" customHeight="1">
-      <c r="A20" s="33" t="inlineStr">
+    <row r="18" ht="56" customHeight="1">
+      <c r="A18" s="33" t="inlineStr">
         <is>
           <t>Field-Assist Agent</t>
         </is>
       </c>
-      <c r="B20" s="18" t="inlineStr">
+      <c r="B18" s="18" t="inlineStr">
         <is>
           <t>MVP 2</t>
         </is>
       </c>
-      <c r="C20" s="18" t="inlineStr">
+      <c r="C18" s="18" t="inlineStr">
         <is>
           <t>Decorator opens new blueprint form — fires when product name + supplier entered</t>
         </is>
       </c>
-      <c r="D20" s="18" t="inlineStr">
+      <c r="D18" s="18" t="inlineStr">
         <is>
           <t>Reads product name + supplier data sheet (PDF/URL). Pre-fills material_tier, tannage_method, finish_type. Decorator reviews and confirms — does not auto-submit.</t>
         </is>
       </c>
-      <c r="E20" s="18" t="inlineStr">
+      <c r="E18" s="18" t="inlineStr">
         <is>
           <t>Form error rate &lt; 10% · Onboarding &lt; 24h</t>
         </is>
       </c>
-      <c r="F20" s="52" t="inlineStr">
+      <c r="F18" s="52" t="inlineStr">
         <is>
           <t>Wrong pre-fill: Decorator trusts it → incorrect material_tier → MAT-001 reject loop</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="5" customHeight="1"/>
-    <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="3" t="inlineStr">
+    <row r="20" ht="5" customHeight="1"/>
+    <row r="21" ht="16" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>3. Channel Integrations (MVP 3 · W17–W24)</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="28" customHeight="1">
-      <c r="A24" s="4" t="inlineStr">
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Channel</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>Weeks</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>Fields mapped</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>Compliance requirement</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="F22" s="4" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>Shopify</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>W17–18</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>material_tier → metafield · tannage_method → metafield · ECO badge</t>
+        </is>
+      </c>
+      <c r="D23" s="10" t="inlineStr">
+        <is>
+          <t>None special</t>
+        </is>
+      </c>
+      <c r="E23" s="10" t="inlineStr"/>
+      <c r="F23" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="33" t="inlineStr">
+        <is>
+          <t>Etsy</t>
+        </is>
+      </c>
+      <c r="B24" s="18" t="inlineStr">
+        <is>
+          <t>W17–18</t>
+        </is>
+      </c>
+      <c r="C24" s="18" t="inlineStr">
+        <is>
+          <t>material_tier → material attribute · handmade_type auto-mapped</t>
+        </is>
+      </c>
+      <c r="D24" s="18" t="inlineStr">
+        <is>
+          <t>None special</t>
+        </is>
+      </c>
+      <c r="E24" s="18" t="inlineStr"/>
+      <c r="F24" s="18" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+    </row>
     <row r="25">
-      <c r="A25" s="9" t="inlineStr">
-        <is>
-          <t>Shopify</t>
-        </is>
-      </c>
-      <c r="B25" s="10" t="inlineStr">
-        <is>
-          <t>W17–18</t>
-        </is>
-      </c>
-      <c r="C25" s="10" t="inlineStr">
-        <is>
-          <t>material_tier → metafield · tannage_method → metafield · ECO badge</t>
-        </is>
-      </c>
-      <c r="D25" s="10" t="inlineStr">
-        <is>
-          <t>None special</t>
-        </is>
-      </c>
-      <c r="E25" s="10" t="inlineStr"/>
-      <c r="F25" s="10" t="inlineStr">
+      <c r="A25" s="56" t="inlineStr">
+        <is>
+          <t>Amazon USA</t>
+        </is>
+      </c>
+      <c r="B25" s="57" t="inlineStr">
+        <is>
+          <t>W19–22</t>
+        </is>
+      </c>
+      <c r="C25" s="57" t="inlineStr">
+        <is>
+          <t>material_tier → LeatherType node · prop_65_compliant → Prop 65 auto-disclosure · chrome → mandatory disclosure</t>
+        </is>
+      </c>
+      <c r="D25" s="57" t="inlineStr">
+        <is>
+          <t>SP-API approval + Prop 65 legal sign-off by W10</t>
+        </is>
+      </c>
+      <c r="E25" s="50" t="inlineStr">
+        <is>
+          <t>⚠ SP-API approval 2–4w — apply W10</t>
+        </is>
+      </c>
+      <c r="F25" s="57" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -8062,17 +8066,17 @@
     <row r="26">
       <c r="A26" s="33" t="inlineStr">
         <is>
-          <t>Etsy</t>
+          <t>WooCommerce</t>
         </is>
       </c>
       <c r="B26" s="18" t="inlineStr">
         <is>
-          <t>W17–18</t>
+          <t>W23–24</t>
         </is>
       </c>
       <c r="C26" s="18" t="inlineStr">
         <is>
-          <t>material_tier → material attribute · handmade_type auto-mapped</t>
+          <t>material_tier + compliance fields → WC product attributes</t>
         </is>
       </c>
       <c r="D26" s="18" t="inlineStr">
@@ -8083,128 +8087,68 @@
       <c r="E26" s="18" t="inlineStr"/>
       <c r="F26" s="18" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="56" t="inlineStr">
-        <is>
-          <t>Amazon USA</t>
-        </is>
-      </c>
-      <c r="B27" s="57" t="inlineStr">
-        <is>
-          <t>W19–22</t>
-        </is>
-      </c>
-      <c r="C27" s="57" t="inlineStr">
-        <is>
-          <t>material_tier → LeatherType node · prop_65_compliant → Prop 65 auto-disclosure · chrome → mandatory disclosure</t>
-        </is>
-      </c>
-      <c r="D27" s="57" t="inlineStr">
-        <is>
-          <t>SP-API approval + Prop 65 legal sign-off by W10</t>
-        </is>
-      </c>
-      <c r="E27" s="50" t="inlineStr">
-        <is>
-          <t>⚠ SP-API approval 2–4w — apply W10</t>
-        </is>
-      </c>
-      <c r="F27" s="57" t="inlineStr">
-        <is>
-          <t>P0</t>
+      <c r="A27" s="110" t="inlineStr">
+        <is>
+          <t>TikTok Shop</t>
+        </is>
+      </c>
+      <c r="B27" s="51" t="inlineStr">
+        <is>
+          <t>V2</t>
+        </is>
+      </c>
+      <c r="C27" s="51" t="inlineStr">
+        <is>
+          <t>Manual disclosure (no API support for leather type yet)</t>
+        </is>
+      </c>
+      <c r="D27" s="51" t="inlineStr">
+        <is>
+          <t>Manual Prop 65 for CA sellers</t>
+        </is>
+      </c>
+      <c r="E27" s="51" t="inlineStr"/>
+      <c r="F27" s="51" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="33" t="inlineStr">
-        <is>
-          <t>WooCommerce</t>
-        </is>
-      </c>
-      <c r="B28" s="18" t="inlineStr">
-        <is>
-          <t>W23–24</t>
-        </is>
-      </c>
-      <c r="C28" s="18" t="inlineStr">
-        <is>
-          <t>material_tier + compliance fields → WC product attributes</t>
-        </is>
-      </c>
-      <c r="D28" s="18" t="inlineStr">
+      <c r="A28" s="111" t="inlineStr">
+        <is>
+          <t>PrestaShop</t>
+        </is>
+      </c>
+      <c r="B28" s="47" t="inlineStr">
+        <is>
+          <t>V2</t>
+        </is>
+      </c>
+      <c r="C28" s="47" t="inlineStr">
+        <is>
+          <t>Custom module (WC plugin base)</t>
+        </is>
+      </c>
+      <c r="D28" s="47" t="inlineStr">
         <is>
           <t>None special</t>
         </is>
       </c>
-      <c r="E28" s="18" t="inlineStr"/>
-      <c r="F28" s="18" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="111" t="inlineStr">
-        <is>
-          <t>TikTok Shop</t>
-        </is>
-      </c>
-      <c r="B29" s="51" t="inlineStr">
-        <is>
-          <t>V2</t>
-        </is>
-      </c>
-      <c r="C29" s="51" t="inlineStr">
-        <is>
-          <t>Manual disclosure (no API support for leather type yet)</t>
-        </is>
-      </c>
-      <c r="D29" s="51" t="inlineStr">
-        <is>
-          <t>Manual Prop 65 for CA sellers</t>
-        </is>
-      </c>
-      <c r="E29" s="51" t="inlineStr"/>
-      <c r="F29" s="51" t="inlineStr">
+      <c r="E28" s="47" t="inlineStr"/>
+      <c r="F28" s="47" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="110" t="inlineStr">
-        <is>
-          <t>PrestaShop</t>
-        </is>
-      </c>
-      <c r="B30" s="47" t="inlineStr">
-        <is>
-          <t>V2</t>
-        </is>
-      </c>
-      <c r="C30" s="47" t="inlineStr">
-        <is>
-          <t>Custom module (WC plugin base)</t>
-        </is>
-      </c>
-      <c r="D30" s="47" t="inlineStr">
-        <is>
-          <t>None special</t>
-        </is>
-      </c>
-      <c r="E30" s="47" t="inlineStr"/>
-      <c r="F30" s="47" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="24" customHeight="1">
-      <c r="A32" s="34" t="inlineStr">
+    <row r="30" ht="24" customHeight="1">
+      <c r="A30" s="34" t="inlineStr">
         <is>
           <t>Amazon is the highest-risk integration: SP-API application must start W10 (2–4w approval) and Prop 65 legal sign-off needed before W19 go-live. PrestaShop and TikTok Shop deferred to V2 — low USA volume relative to Shopify/Etsy/Amazon.</t>
         </is>
@@ -8212,11 +8156,11 @@
     </row>
   </sheetData>
   <mergeCells count="5">
+    <mergeCell ref="A30:F30"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A23:F23"/>
-    <mergeCell ref="A32:F32"/>
-    <mergeCell ref="A17:F17"/>
     <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A21:F21"/>
+    <mergeCell ref="A15:F15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Excel: white section bars + References section in Business Case
- Section bars: #3D6B28 → white background, dark green text (readable, clean)
- Business Case tab: new section 7 — Sources & References with 8 clickable links
  Nova One Advisor · accio.com · eRank · ShelfTrend · Shopify · FTC · PrintKK · GitHub

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/Printify_Leather_PRD_Workbook.xlsx
+++ b/output/Printify_Leather_PRD_Workbook.xlsx
@@ -49,7 +49,7 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="002B5A18"/>
       <sz val="10"/>
     </font>
     <font>
@@ -146,7 +146,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -155,7 +155,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="003D6B28"/>
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -171,11 +171,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E4FCC0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -289,7 +284,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="112">
+  <cellXfs count="114">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -339,19 +334,19 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -378,216 +373,222 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="14" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="14" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="14" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="14" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -599,15 +600,15 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -4499,7 +4500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G81"/>
+  <dimension ref="A1:G93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5810,25 +5811,241 @@
         </is>
       </c>
     </row>
+    <row r="83" ht="5" customHeight="1"/>
+    <row r="84" ht="16" customHeight="1">
+      <c r="A84" s="3" t="inlineStr">
+        <is>
+          <t>7. Sources &amp; References</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="28" customHeight="1">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>Data point used</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr"/>
+      <c r="E85" s="4" t="inlineStr"/>
+      <c r="F85" s="4" t="inlineStr"/>
+      <c r="G85" s="4" t="inlineStr"/>
+    </row>
+    <row r="86" ht="20" customHeight="1">
+      <c r="A86" s="9" t="inlineStr">
+        <is>
+          <t>Nova One Advisor 2025</t>
+        </is>
+      </c>
+      <c r="B86" s="10" t="inlineStr">
+        <is>
+          <t>US leather goods market: $54.26B TAM · 6.7% CAGR</t>
+        </is>
+      </c>
+      <c r="C86" s="100" t="inlineStr">
+        <is>
+          <t>https://www.novaoneadvisor.com/report/us-leather-goods-market</t>
+        </is>
+      </c>
+      <c r="D86" s="36" t="n"/>
+      <c r="E86" s="36" t="n"/>
+      <c r="F86" s="36" t="n"/>
+      <c r="G86" s="37" t="n"/>
+    </row>
+    <row r="87" ht="20" customHeight="1">
+      <c r="A87" s="33" t="inlineStr">
+        <is>
+          <t>accio.com 2025</t>
+        </is>
+      </c>
+      <c r="B87" s="18" t="inlineStr">
+        <is>
+          <t>Amazon USA BSR: BULLIANT leather wallet — 8,365 units/month</t>
+        </is>
+      </c>
+      <c r="C87" s="101" t="inlineStr">
+        <is>
+          <t>https://www.accio.com/business/amazon-mens-wallet-best-seller</t>
+        </is>
+      </c>
+      <c r="D87" s="36" t="n"/>
+      <c r="E87" s="36" t="n"/>
+      <c r="F87" s="36" t="n"/>
+      <c r="G87" s="37" t="n"/>
+    </row>
+    <row r="88" ht="20" customHeight="1">
+      <c r="A88" s="9" t="inlineStr">
+        <is>
+          <t>eRank 2025</t>
+        </is>
+      </c>
+      <c r="B88" s="10" t="inlineStr">
+        <is>
+          <t>Etsy USA: "leather" = #215 top keyword · +57% search growth Nov–Dec</t>
+        </is>
+      </c>
+      <c r="C88" s="100" t="inlineStr">
+        <is>
+          <t>https://erank.com</t>
+        </is>
+      </c>
+      <c r="D88" s="36" t="n"/>
+      <c r="E88" s="36" t="n"/>
+      <c r="F88" s="36" t="n"/>
+      <c r="G88" s="37" t="n"/>
+    </row>
+    <row r="89" ht="20" customHeight="1">
+      <c r="A89" s="33" t="inlineStr">
+        <is>
+          <t>ShelfTrend 2025</t>
+        </is>
+      </c>
+      <c r="B89" s="18" t="inlineStr">
+        <is>
+          <t>Etsy top-quartile leather sellers: 15–25 orders/SKU/mo · "personalized leather bag" GMV $130K–$270K/week</t>
+        </is>
+      </c>
+      <c r="C89" s="101" t="inlineStr">
+        <is>
+          <t>https://shelftrend.com</t>
+        </is>
+      </c>
+      <c r="D89" s="36" t="n"/>
+      <c r="E89" s="36" t="n"/>
+      <c r="F89" s="36" t="n"/>
+      <c r="G89" s="37" t="n"/>
+    </row>
+    <row r="90" ht="20" customHeight="1">
+      <c r="A90" s="9" t="inlineStr">
+        <is>
+          <t>Shopify Materials Attributes (2025)</t>
+        </is>
+      </c>
+      <c r="B90" s="10" t="inlineStr">
+        <is>
+          <t>New material attribute standard enabling leather taxonomy in Shopify metafields — no indexing lag</t>
+        </is>
+      </c>
+      <c r="C90" s="100" t="inlineStr">
+        <is>
+          <t>https://help.shopify.com/en/manual/products/details/product-type</t>
+        </is>
+      </c>
+      <c r="D90" s="36" t="n"/>
+      <c r="E90" s="36" t="n"/>
+      <c r="F90" s="36" t="n"/>
+      <c r="G90" s="37" t="n"/>
+    </row>
+    <row r="91" ht="20" customHeight="1">
+      <c r="A91" s="33" t="inlineStr">
+        <is>
+          <t>FTC Guides for Textile &amp; Fur (MAT-001)</t>
+        </is>
+      </c>
+      <c r="B91" s="18" t="inlineStr">
+        <is>
+          <t>Genuine leather labeling requirements · PU/bonded cannot be labeled "genuine leather"</t>
+        </is>
+      </c>
+      <c r="C91" s="101" t="inlineStr">
+        <is>
+          <t>https://www.ftc.gov/legal-library/browse/rules/guides-use-word-leather</t>
+        </is>
+      </c>
+      <c r="D91" s="36" t="n"/>
+      <c r="E91" s="36" t="n"/>
+      <c r="F91" s="36" t="n"/>
+      <c r="G91" s="37" t="n"/>
+    </row>
+    <row r="92" ht="20" customHeight="1">
+      <c r="A92" s="9" t="inlineStr">
+        <is>
+          <t>PrintKK (public catalog)</t>
+        </is>
+      </c>
+      <c r="B92" s="10" t="inlineStr">
+        <is>
+          <t>Competitor genuine leather POD: 50-unit MOQ · no taxonomy · no FTC compliance</t>
+        </is>
+      </c>
+      <c r="C92" s="100" t="inlineStr">
+        <is>
+          <t>https://printkk.com</t>
+        </is>
+      </c>
+      <c r="D92" s="36" t="n"/>
+      <c r="E92" s="36" t="n"/>
+      <c r="F92" s="36" t="n"/>
+      <c r="G92" s="37" t="n"/>
+    </row>
+    <row r="93" ht="20" customHeight="1">
+      <c r="A93" s="33" t="inlineStr">
+        <is>
+          <t>GitHub — Full PRD &amp; financial model</t>
+        </is>
+      </c>
+      <c r="B93" s="18" t="inlineStr">
+        <is>
+          <t>All deliverables: PRD HTML, Excel workbook, demand charts, interview prep</t>
+        </is>
+      </c>
+      <c r="C93" s="101" t="inlineStr">
+        <is>
+          <t>https://github.com/elenacastan-maker/fyul-pm-interview-prep</t>
+        </is>
+      </c>
+      <c r="D93" s="36" t="n"/>
+      <c r="E93" s="36" t="n"/>
+      <c r="F93" s="36" t="n"/>
+      <c r="G93" s="37" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="23">
+    <mergeCell ref="C92:G92"/>
+    <mergeCell ref="C86:G86"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="C89:G89"/>
+    <mergeCell ref="A81:G81"/>
+    <mergeCell ref="C88:G88"/>
     <mergeCell ref="A13:G13"/>
-    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A40:G40"/>
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A6:G6"/>
     <mergeCell ref="A34:G34"/>
-    <mergeCell ref="A4:G4"/>
     <mergeCell ref="A24:G24"/>
-    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="C93:G93"/>
     <mergeCell ref="A15:G15"/>
     <mergeCell ref="A64:G64"/>
+    <mergeCell ref="C90:G90"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A6:G6"/>
     <mergeCell ref="A25:G25"/>
-    <mergeCell ref="A81:G81"/>
+    <mergeCell ref="A84:G84"/>
+    <mergeCell ref="C91:G91"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A2:G2"/>
     <mergeCell ref="A71:G71"/>
+    <mergeCell ref="C87:G87"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C86" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C87" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C88" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C89" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C90" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C91" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C92" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C93" r:id="rId8"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9"/>
 </worksheet>
 </file>
 
@@ -5919,7 +6136,7 @@
           <t>❌ 0</t>
         </is>
       </c>
-      <c r="C5" s="100" t="inlineStr">
+      <c r="C5" s="102" t="inlineStr">
         <is>
           <t>✅ 150+ SKUs</t>
         </is>
@@ -5961,7 +6178,7 @@
           <t>✅ ~45</t>
         </is>
       </c>
-      <c r="C6" s="100" t="inlineStr">
+      <c r="C6" s="102" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -6003,7 +6220,7 @@
           <t>❌</t>
         </is>
       </c>
-      <c r="C7" s="100" t="inlineStr">
+      <c r="C7" s="102" t="inlineStr">
         <is>
           <t>✅ 8 fields</t>
         </is>
@@ -6045,7 +6262,7 @@
           <t>❌</t>
         </is>
       </c>
-      <c r="C8" s="100" t="inlineStr">
+      <c r="C8" s="102" t="inlineStr">
         <is>
           <t>✅ MAT-001</t>
         </is>
@@ -6087,7 +6304,7 @@
           <t>❌</t>
         </is>
       </c>
-      <c r="C9" s="100" t="inlineStr">
+      <c r="C9" s="102" t="inlineStr">
         <is>
           <t>✅ MVP 1</t>
         </is>
@@ -6129,7 +6346,7 @@
           <t>❌</t>
         </is>
       </c>
-      <c r="C10" s="100" t="inlineStr">
+      <c r="C10" s="102" t="inlineStr">
         <is>
           <t>✅ MVP 1</t>
         </is>
@@ -6171,7 +6388,7 @@
           <t>❌</t>
         </is>
       </c>
-      <c r="C11" s="100" t="inlineStr">
+      <c r="C11" s="102" t="inlineStr">
         <is>
           <t>✅ MVP 2</t>
         </is>
@@ -6213,7 +6430,7 @@
           <t>❌</t>
         </is>
       </c>
-      <c r="C12" s="100" t="inlineStr">
+      <c r="C12" s="102" t="inlineStr">
         <is>
           <t>✅ MVP 2</t>
         </is>
@@ -6255,7 +6472,7 @@
           <t>❌</t>
         </is>
       </c>
-      <c r="C13" s="100" t="inlineStr">
+      <c r="C13" s="102" t="inlineStr">
         <is>
           <t>✅ MVP 2</t>
         </is>
@@ -6297,7 +6514,7 @@
           <t>❌</t>
         </is>
       </c>
-      <c r="C14" s="100" t="inlineStr">
+      <c r="C14" s="102" t="inlineStr">
         <is>
           <t>✅ MVP 3</t>
         </is>
@@ -6339,7 +6556,7 @@
           <t>❌</t>
         </is>
       </c>
-      <c r="C15" s="100" t="inlineStr">
+      <c r="C15" s="102" t="inlineStr">
         <is>
           <t>✅ MVP 3</t>
         </is>
@@ -6381,7 +6598,7 @@
           <t>❌</t>
         </is>
       </c>
-      <c r="C16" s="101" t="inlineStr">
+      <c r="C16" s="103" t="inlineStr">
         <is>
           <t>⏳ V2</t>
         </is>
@@ -6423,7 +6640,7 @@
           <t>⚠ Generic</t>
         </is>
       </c>
-      <c r="C17" s="100" t="inlineStr">
+      <c r="C17" s="102" t="inlineStr">
         <is>
           <t>✅ MVP 3</t>
         </is>
@@ -6975,196 +7192,196 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="102" t="inlineStr">
+      <c r="A13" s="104" t="inlineStr">
         <is>
           <t>Phase</t>
         </is>
       </c>
-      <c r="B13" s="103" t="inlineStr">
+      <c r="B13" s="105" t="inlineStr">
         <is>
           <t>W0</t>
         </is>
       </c>
-      <c r="C13" s="103" t="inlineStr">
+      <c r="C13" s="105" t="inlineStr">
         <is>
           <t>W1</t>
         </is>
       </c>
-      <c r="D13" s="103" t="inlineStr">
+      <c r="D13" s="105" t="inlineStr">
         <is>
           <t>W2</t>
         </is>
       </c>
-      <c r="E13" s="103" t="inlineStr">
+      <c r="E13" s="105" t="inlineStr">
         <is>
           <t>W3</t>
         </is>
       </c>
-      <c r="F13" s="103" t="inlineStr">
+      <c r="F13" s="105" t="inlineStr">
         <is>
           <t>W4</t>
         </is>
       </c>
-      <c r="G13" s="103" t="inlineStr">
+      <c r="G13" s="105" t="inlineStr">
         <is>
           <t>W5</t>
         </is>
       </c>
-      <c r="H13" s="103" t="inlineStr">
+      <c r="H13" s="105" t="inlineStr">
         <is>
           <t>W6</t>
         </is>
       </c>
-      <c r="I13" s="103" t="inlineStr">
+      <c r="I13" s="105" t="inlineStr">
         <is>
           <t>W7</t>
         </is>
       </c>
-      <c r="J13" s="103" t="inlineStr">
+      <c r="J13" s="105" t="inlineStr">
         <is>
           <t>W8</t>
         </is>
       </c>
-      <c r="K13" s="103" t="inlineStr">
+      <c r="K13" s="105" t="inlineStr">
         <is>
           <t>W9</t>
         </is>
       </c>
-      <c r="L13" s="103" t="inlineStr">
+      <c r="L13" s="105" t="inlineStr">
         <is>
           <t>W10</t>
         </is>
       </c>
-      <c r="M13" s="103" t="inlineStr">
+      <c r="M13" s="105" t="inlineStr">
         <is>
           <t>W11</t>
         </is>
       </c>
-      <c r="N13" s="103" t="inlineStr">
+      <c r="N13" s="105" t="inlineStr">
         <is>
           <t>W12</t>
         </is>
       </c>
-      <c r="O13" s="103" t="inlineStr">
+      <c r="O13" s="105" t="inlineStr">
         <is>
           <t>W13</t>
         </is>
       </c>
-      <c r="P13" s="103" t="inlineStr">
+      <c r="P13" s="105" t="inlineStr">
         <is>
           <t>W14</t>
         </is>
       </c>
-      <c r="Q13" s="103" t="inlineStr">
+      <c r="Q13" s="105" t="inlineStr">
         <is>
           <t>W15</t>
         </is>
       </c>
-      <c r="R13" s="103" t="inlineStr">
+      <c r="R13" s="105" t="inlineStr">
         <is>
           <t>W16</t>
         </is>
       </c>
-      <c r="S13" s="103" t="inlineStr">
+      <c r="S13" s="105" t="inlineStr">
         <is>
           <t>W17</t>
         </is>
       </c>
-      <c r="T13" s="103" t="inlineStr">
+      <c r="T13" s="105" t="inlineStr">
         <is>
           <t>W18</t>
         </is>
       </c>
-      <c r="U13" s="103" t="inlineStr">
+      <c r="U13" s="105" t="inlineStr">
         <is>
           <t>W19</t>
         </is>
       </c>
-      <c r="V13" s="103" t="inlineStr">
+      <c r="V13" s="105" t="inlineStr">
         <is>
           <t>W20</t>
         </is>
       </c>
-      <c r="W13" s="103" t="inlineStr">
+      <c r="W13" s="105" t="inlineStr">
         <is>
           <t>W21</t>
         </is>
       </c>
-      <c r="X13" s="103" t="inlineStr">
+      <c r="X13" s="105" t="inlineStr">
         <is>
           <t>W22</t>
         </is>
       </c>
-      <c r="Y13" s="103" t="inlineStr">
+      <c r="Y13" s="105" t="inlineStr">
         <is>
           <t>W23</t>
         </is>
       </c>
-      <c r="Z13" s="103" t="inlineStr">
+      <c r="Z13" s="105" t="inlineStr">
         <is>
           <t>W24</t>
         </is>
       </c>
     </row>
     <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="104" t="inlineStr">
+      <c r="A14" s="106" t="inlineStr">
         <is>
           <t>PoC</t>
         </is>
       </c>
-      <c r="B14" s="105" t="n"/>
+      <c r="B14" s="107" t="n"/>
     </row>
     <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="104" t="inlineStr">
+      <c r="A15" s="106" t="inlineStr">
         <is>
           <t>Design Sprint</t>
         </is>
       </c>
-      <c r="C15" s="106" t="n"/>
-      <c r="D15" s="106" t="n"/>
+      <c r="C15" s="108" t="n"/>
+      <c r="D15" s="108" t="n"/>
     </row>
     <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="104" t="inlineStr">
+      <c r="A16" s="106" t="inlineStr">
         <is>
           <t>MVP 1 — Schema</t>
         </is>
       </c>
-      <c r="E16" s="107" t="n"/>
-      <c r="F16" s="107" t="n"/>
-      <c r="G16" s="107" t="n"/>
-      <c r="H16" s="107" t="n"/>
-      <c r="I16" s="107" t="n"/>
-      <c r="J16" s="107" t="n"/>
+      <c r="E16" s="109" t="n"/>
+      <c r="F16" s="109" t="n"/>
+      <c r="G16" s="109" t="n"/>
+      <c r="H16" s="109" t="n"/>
+      <c r="I16" s="109" t="n"/>
+      <c r="J16" s="109" t="n"/>
     </row>
     <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="104" t="inlineStr">
+      <c r="A17" s="106" t="inlineStr">
         <is>
           <t>MVP 2 — Mockup</t>
         </is>
       </c>
-      <c r="K17" s="108" t="n"/>
-      <c r="L17" s="108" t="n"/>
-      <c r="M17" s="108" t="n"/>
-      <c r="N17" s="108" t="n"/>
-      <c r="O17" s="108" t="n"/>
-      <c r="P17" s="108" t="n"/>
-      <c r="Q17" s="108" t="n"/>
-      <c r="R17" s="108" t="n"/>
+      <c r="K17" s="110" t="n"/>
+      <c r="L17" s="110" t="n"/>
+      <c r="M17" s="110" t="n"/>
+      <c r="N17" s="110" t="n"/>
+      <c r="O17" s="110" t="n"/>
+      <c r="P17" s="110" t="n"/>
+      <c r="Q17" s="110" t="n"/>
+      <c r="R17" s="110" t="n"/>
     </row>
     <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="104" t="inlineStr">
+      <c r="A18" s="106" t="inlineStr">
         <is>
           <t>MVP 3 — Channels</t>
         </is>
       </c>
-      <c r="S18" s="109" t="n"/>
-      <c r="T18" s="109" t="n"/>
-      <c r="U18" s="109" t="n"/>
-      <c r="V18" s="109" t="n"/>
-      <c r="W18" s="109" t="n"/>
-      <c r="X18" s="109" t="n"/>
-      <c r="Y18" s="109" t="n"/>
-      <c r="Z18" s="109" t="n"/>
+      <c r="S18" s="111" t="n"/>
+      <c r="T18" s="111" t="n"/>
+      <c r="U18" s="111" t="n"/>
+      <c r="V18" s="111" t="n"/>
+      <c r="W18" s="111" t="n"/>
+      <c r="X18" s="111" t="n"/>
+      <c r="Y18" s="111" t="n"/>
+      <c r="Z18" s="111" t="n"/>
     </row>
     <row r="21" customHeight="1">
       <c r="A21" t="inlineStr">
@@ -8092,7 +8309,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="110" t="inlineStr">
+      <c r="A27" s="112" t="inlineStr">
         <is>
           <t>TikTok Shop</t>
         </is>
@@ -8120,7 +8337,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="111" t="inlineStr">
+      <c r="A28" s="113" t="inlineStr">
         <is>
           <t>PrestaShop</t>
         </is>

</xml_diff>